<commit_message>
Add fields to shipping request template
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/선적 요청_템플릿.xlsx
+++ b/선적 요청_템플릿.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\8. ATA CARNET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E67742E8-B20E-401D-9587-8349628EC187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A6D777A-B611-4236-9080-821DF47933D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{E8EE0F76-5C41-4E3B-8CCB-DD9C80B10C1A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="60">
   <si>
     <t>선적 방식</t>
   </si>
@@ -406,13 +406,46 @@
 - TPU, PC, neodymium, PLA, 배터리 포함</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>담당자 정보</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>까르네 사용자</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>해당 증서를 제출하고 
+통관업무를 진행할 담당자</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>내부 프로세스</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예산&amp;지출결의 품의</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>비밀유지 계약서</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>○○팀, ○○○과장</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>담당자명 국문(여권 영문명 기재) : 홍길동 (HONG GILDONG)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="184" formatCode="&quot;USD &quot;#,##0.00"/>
+    <numFmt numFmtId="176" formatCode="&quot;USD &quot;#,##0.00"/>
   </numFmts>
   <fonts count="19" x14ac:knownFonts="1">
     <font>
@@ -663,7 +696,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -709,56 +742,62 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="176" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="184" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1094,7 +1133,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7485E108-DB65-4BD8-8918-0481D713ADE3}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17.4140625" customWidth="1"/>
@@ -1105,35 +1144,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="25"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="27"/>
     </row>
     <row r="3" spans="1:5" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="28"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="30"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="6"/>
@@ -1159,8 +1198,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A6" s="18" t="s">
+    <row r="6" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A6" s="20" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="7" t="s">
@@ -1174,8 +1213,8 @@
       </c>
       <c r="E6" s="9"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A7" s="19"/>
+    <row r="7" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="21"/>
       <c r="B7" s="7" t="s">
         <v>11</v>
       </c>
@@ -1187,8 +1226,8 @@
       </c>
       <c r="E7" s="9"/>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A8" s="19"/>
+    <row r="8" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A8" s="21"/>
       <c r="B8" s="10" t="s">
         <v>43</v>
       </c>
@@ -1200,8 +1239,8 @@
       </c>
       <c r="E8" s="9"/>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A9" s="20"/>
+    <row r="9" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A9" s="22"/>
       <c r="B9" s="7" t="s">
         <v>12</v>
       </c>
@@ -1215,8 +1254,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="26" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="15" t="s">
+    <row r="10" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A10" s="18" t="s">
         <v>14</v>
       </c>
       <c r="B10" s="7" t="s">
@@ -1230,8 +1269,8 @@
       </c>
       <c r="E10" s="9"/>
     </row>
-    <row r="11" spans="1:5" ht="29" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="16"/>
+    <row r="11" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="19"/>
       <c r="B11" s="7" t="s">
         <v>15</v>
       </c>
@@ -1243,8 +1282,8 @@
       </c>
       <c r="E11" s="9"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A12" s="18" t="s">
+    <row r="12" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A12" s="20" t="s">
         <v>33</v>
       </c>
       <c r="B12" s="7" t="s">
@@ -1258,8 +1297,8 @@
       </c>
       <c r="E12" s="9"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A13" s="19"/>
+    <row r="13" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="21"/>
       <c r="B13" s="7" t="s">
         <v>18</v>
       </c>
@@ -1271,30 +1310,34 @@
       </c>
       <c r="E13" s="9"/>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A14" s="19"/>
+    <row r="14" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="21"/>
       <c r="B14" s="10" t="s">
         <v>38</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="2"/>
+      <c r="D14" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="E14" s="9"/>
     </row>
-    <row r="15" spans="1:5" ht="31.5" x14ac:dyDescent="0.45">
-      <c r="A15" s="20"/>
+    <row r="15" spans="1:5" ht="39" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="22"/>
       <c r="B15" s="12" t="s">
         <v>39</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="D15" s="2"/>
+      <c r="D15" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="E15" s="9"/>
     </row>
     <row r="16" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="18" t="s">
         <v>20</v>
       </c>
       <c r="B16" s="7" t="s">
@@ -1310,12 +1353,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="17"/>
+    <row r="17" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="31"/>
       <c r="B17" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="31" t="s">
+      <c r="C17" s="17" t="s">
         <v>51</v>
       </c>
       <c r="D17" s="2" t="s">
@@ -1325,8 +1368,8 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A18" s="17"/>
+    <row r="18" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="31"/>
       <c r="B18" s="13" t="s">
         <v>44</v>
       </c>
@@ -1338,64 +1381,103 @@
       </c>
       <c r="E18" s="9"/>
     </row>
-    <row r="19" spans="1:5" ht="29" x14ac:dyDescent="0.45">
-      <c r="A19" s="17"/>
+    <row r="19" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="31"/>
       <c r="B19" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="C19" s="29">
+      <c r="C19" s="15">
         <v>100</v>
       </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="30" t="s">
+      <c r="D19" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E19" s="16" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A20" s="16"/>
+    <row r="20" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="19"/>
       <c r="B20" s="14" t="s">
         <v>45</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D20" s="2"/>
-      <c r="E20" s="30" t="s">
+      <c r="D20" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E20" s="16" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A21" s="15" t="s">
+    <row r="21" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E21" s="16" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A22" s="33"/>
+      <c r="B22" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E22" s="16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B23" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C23" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E21" s="9"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A22" s="16"/>
-      <c r="B22" s="7" t="s">
+      <c r="D23" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" s="16" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A24" s="19"/>
+      <c r="B24" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C24" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="D24" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E22" s="9"/>
+      <c r="E24" s="9"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A21:A22"/>
     <mergeCell ref="A10:A11"/>
-    <mergeCell ref="A21:A22"/>
     <mergeCell ref="A12:A15"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="B2:E2"/>

</xml_diff>

<commit_message>
Reorder shipping request template categories (product info first)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/선적 요청_템플릿.xlsx
+++ b/선적 요청_템플릿.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\8. ATA CARNET\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A6D777A-B611-4236-9080-821DF47933D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FE9E259-0B2A-4933-9492-F2C6E289238B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{E8EE0F76-5C41-4E3B-8CCB-DD9C80B10C1A}"/>
   </bookViews>
@@ -48,9 +48,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>수출 관련 정보 수집 요청</t>
-  </si>
-  <si>
     <t>카테고리</t>
   </si>
   <si>
@@ -437,6 +434,83 @@
   </si>
   <si>
     <t>담당자명 국문(여권 영문명 기재) : 홍길동 (HONG GILDONG)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수출</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>관련</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>정보 확인</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>요청</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -447,7 +521,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="&quot;USD &quot;#,##0.00"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -578,6 +652,22 @@
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
   </fonts>
   <fills count="5">
@@ -757,6 +847,12 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -766,9 +862,6 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -793,11 +886,8 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1144,35 +1234,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="23" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
+      <c r="A1" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="27"/>
+        <v>29</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="28"/>
     </row>
     <row r="3" spans="1:5" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="28" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30"/>
+        <v>49</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="31"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="6"/>
@@ -1183,293 +1273,293 @@
     </row>
     <row r="5" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="6" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="20" t="s">
-        <v>1</v>
+      <c r="A6" s="18" t="s">
+        <v>19</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="9"/>
-    </row>
-    <row r="7" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A7" s="21"/>
-      <c r="B7" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>10</v>
+        <v>7</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="32"/>
+      <c r="B7" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>50</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="9"/>
+        <v>7</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="8" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A8" s="21"/>
-      <c r="B8" s="10" t="s">
+      <c r="A8" s="32"/>
+      <c r="B8" s="13" t="s">
         <v>43</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8" s="9"/>
     </row>
     <row r="9" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" s="22"/>
-      <c r="B9" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>42</v>
+      <c r="A9" s="32"/>
+      <c r="B9" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="15">
+        <v>100</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A10" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>0</v>
+      <c r="A10" s="19"/>
+      <c r="B10" s="14" t="s">
+        <v>44</v>
       </c>
       <c r="C10" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A11" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="9"/>
-    </row>
-    <row r="11" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A11" s="19"/>
-      <c r="B11" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>16</v>
-      </c>
       <c r="D11" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E11" s="9"/>
     </row>
     <row r="12" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="20" t="s">
-        <v>33</v>
-      </c>
+      <c r="A12" s="23"/>
       <c r="B12" s="7" t="s">
         <v>17</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E12" s="9"/>
     </row>
     <row r="13" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A13" s="21"/>
-      <c r="B13" s="7" t="s">
-        <v>18</v>
+      <c r="A13" s="23"/>
+      <c r="B13" s="10" t="s">
+        <v>37</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E13" s="9"/>
     </row>
-    <row r="14" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="21"/>
-      <c r="B14" s="10" t="s">
+    <row r="14" spans="1:5" ht="39" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="24"/>
+      <c r="B14" s="12" t="s">
         <v>38</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>40</v>
       </c>
       <c r="D14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="9"/>
+    </row>
+    <row r="15" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="9"/>
+    </row>
+    <row r="16" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="19"/>
+      <c r="B16" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="9"/>
+    </row>
+    <row r="17" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="22" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="9"/>
-    </row>
-    <row r="15" spans="1:5" ht="39" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="22"/>
-      <c r="B15" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="8" t="s">
+      <c r="C17" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" s="9"/>
+    </row>
+    <row r="18" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="23"/>
+      <c r="B18" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" s="9"/>
+    </row>
+    <row r="19" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="23"/>
+      <c r="B19" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E19" s="9"/>
+    </row>
+    <row r="20" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="24"/>
+      <c r="B20" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" s="9"/>
-    </row>
-    <row r="16" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="58" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="31"/>
-      <c r="B17" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" s="17" t="s">
+    </row>
+    <row r="21" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="20" t="s">
         <v>51</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="31"/>
-      <c r="B18" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E18" s="9"/>
-    </row>
-    <row r="19" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="31"/>
-      <c r="B19" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C19" s="15">
-        <v>100</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E19" s="16" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="19"/>
-      <c r="B20" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E20" s="16" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="32" t="s">
+      <c r="B21" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="C21" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E21" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="C21" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E21" s="16" t="s">
+    </row>
+    <row r="22" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A22" s="21"/>
+      <c r="B22" s="14" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="33"/>
-      <c r="B22" s="14" t="s">
+      <c r="C22" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E22" s="16" t="s">
         <v>55</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="C23" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="8" t="s">
-        <v>27</v>
-      </c>
       <c r="D23" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E23" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="27" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="19"/>
       <c r="B24" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C24" s="8" t="s">
-        <v>29</v>
-      </c>
       <c r="D24" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E24" s="9"/>
     </row>
@@ -1477,13 +1567,13 @@
   <mergeCells count="9">
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A11:A14"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="B3:E3"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A16:A20"/>
+    <mergeCell ref="A17:A20"/>
+    <mergeCell ref="A6:A10"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>